<commit_message>
Rename Week → Part in Eddie's remediation plan
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/eddie/custom-mobymax-reading-plan.xlsx
+++ b/eddie/custom-mobymax-reading-plan.xlsx
@@ -560,7 +560,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Week</t>
+          <t>Part</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -597,14 +597,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Week 1: Inference &amp; Evidence Foundations</t>
+          <t>Part 1: Inference &amp; Evidence Foundations</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Week 1</t>
+          <t>Part 1</t>
         </is>
       </c>
       <c r="B3" s="4" t="n">
@@ -637,7 +637,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Week 1</t>
+          <t>Part 1</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
@@ -670,7 +670,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Week 1</t>
+          <t>Part 1</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
@@ -703,7 +703,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Week 1</t>
+          <t>Part 1</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
@@ -736,7 +736,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Week 1</t>
+          <t>Part 1</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
@@ -769,7 +769,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Week 1</t>
+          <t>Part 1</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
@@ -802,7 +802,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Week 1</t>
+          <t>Part 1</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
@@ -835,7 +835,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Week 1</t>
+          <t>Part 1</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
@@ -868,7 +868,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Week 1</t>
+          <t>Part 1</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
@@ -901,7 +901,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Week 1</t>
+          <t>Part 1</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
@@ -934,7 +934,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Week 1</t>
+          <t>Part 1</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
@@ -967,7 +967,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Week 1</t>
+          <t>Part 1</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
@@ -1000,14 +1000,14 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Week 2: Inference &amp; Evidence Mastery</t>
+          <t>Part 2: Inference &amp; Evidence Mastery</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Week 2</t>
+          <t>Part 2</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
@@ -1040,7 +1040,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Week 2</t>
+          <t>Part 2</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
@@ -1073,7 +1073,7 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Week 2</t>
+          <t>Part 2</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
@@ -1106,7 +1106,7 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Week 2</t>
+          <t>Part 2</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
@@ -1139,7 +1139,7 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Week 2</t>
+          <t>Part 2</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
@@ -1172,7 +1172,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Week 2</t>
+          <t>Part 2</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
@@ -1205,7 +1205,7 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Week 2</t>
+          <t>Part 2</t>
         </is>
       </c>
       <c r="B22" s="4" t="n">
@@ -1238,7 +1238,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Week 2</t>
+          <t>Part 2</t>
         </is>
       </c>
       <c r="B23" s="4" t="n">
@@ -1271,7 +1271,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Week 2</t>
+          <t>Part 2</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
@@ -1304,7 +1304,7 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Week 2</t>
+          <t>Part 2</t>
         </is>
       </c>
       <c r="B25" s="4" t="n">
@@ -1337,7 +1337,7 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Week 2</t>
+          <t>Part 2</t>
         </is>
       </c>
       <c r="B26" s="4" t="n">
@@ -1370,7 +1370,7 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Week 2</t>
+          <t>Part 2</t>
         </is>
       </c>
       <c r="B27" s="4" t="n">
@@ -1403,7 +1403,7 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Week 2</t>
+          <t>Part 2</t>
         </is>
       </c>
       <c r="B28" s="4" t="n">
@@ -1436,7 +1436,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Week 2</t>
+          <t>Part 2</t>
         </is>
       </c>
       <c r="B29" s="4" t="n">
@@ -1469,7 +1469,7 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Week 2</t>
+          <t>Part 2</t>
         </is>
       </c>
       <c r="B30" s="4" t="n">
@@ -1502,7 +1502,7 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Week 2</t>
+          <t>Part 2</t>
         </is>
       </c>
       <c r="B31" s="4" t="n">
@@ -1535,14 +1535,14 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Week 3: Author's Purpose &amp; Rhetoric</t>
+          <t>Part 3: Author's Purpose &amp; Rhetoric</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B33" s="4" t="n">
@@ -1575,7 +1575,7 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B34" s="4" t="n">
@@ -1608,7 +1608,7 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B35" s="4" t="n">
@@ -1641,7 +1641,7 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B36" s="4" t="n">
@@ -1674,7 +1674,7 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B37" s="4" t="n">
@@ -1707,7 +1707,7 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B38" s="4" t="n">
@@ -1740,7 +1740,7 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B39" s="4" t="n">
@@ -1773,7 +1773,7 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B40" s="4" t="n">
@@ -1806,7 +1806,7 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B41" s="4" t="n">
@@ -1839,7 +1839,7 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B42" s="4" t="n">
@@ -1872,7 +1872,7 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B43" s="4" t="n">
@@ -1905,7 +1905,7 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B44" s="4" t="n">
@@ -1938,7 +1938,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B45" s="4" t="n">
@@ -1971,7 +1971,7 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B46" s="4" t="n">
@@ -2004,7 +2004,7 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B47" s="4" t="n">
@@ -2037,7 +2037,7 @@
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B48" s="4" t="n">
@@ -2070,7 +2070,7 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B49" s="4" t="n">
@@ -2103,7 +2103,7 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B50" s="4" t="n">
@@ -2136,7 +2136,7 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B51" s="4" t="n">
@@ -2169,7 +2169,7 @@
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B52" s="4" t="n">
@@ -2202,7 +2202,7 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B53" s="4" t="n">
@@ -2235,7 +2235,7 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B54" s="4" t="n">
@@ -2268,7 +2268,7 @@
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B55" s="4" t="n">
@@ -2301,7 +2301,7 @@
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B56" s="4" t="n">
@@ -2334,7 +2334,7 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B57" s="4" t="n">
@@ -2367,7 +2367,7 @@
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B58" s="4" t="n">
@@ -2400,7 +2400,7 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B59" s="4" t="n">
@@ -2433,7 +2433,7 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B60" s="4" t="n">
@@ -2466,7 +2466,7 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B61" s="4" t="n">
@@ -2499,14 +2499,14 @@
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>Week 4: Vocabulary &amp; Context Clues</t>
+          <t>Part 4: Vocabulary &amp; Context Clues</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Week 4</t>
+          <t>Part 4</t>
         </is>
       </c>
       <c r="B63" s="4" t="n">
@@ -2539,7 +2539,7 @@
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>Week 4</t>
+          <t>Part 4</t>
         </is>
       </c>
       <c r="B64" s="4" t="n">
@@ -2572,7 +2572,7 @@
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>Week 4</t>
+          <t>Part 4</t>
         </is>
       </c>
       <c r="B65" s="4" t="n">
@@ -2605,7 +2605,7 @@
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>Week 4</t>
+          <t>Part 4</t>
         </is>
       </c>
       <c r="B66" s="4" t="n">
@@ -2638,7 +2638,7 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>Week 4</t>
+          <t>Part 4</t>
         </is>
       </c>
       <c r="B67" s="4" t="n">
@@ -2671,7 +2671,7 @@
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>Week 4</t>
+          <t>Part 4</t>
         </is>
       </c>
       <c r="B68" s="4" t="n">
@@ -2704,7 +2704,7 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Week 4</t>
+          <t>Part 4</t>
         </is>
       </c>
       <c r="B69" s="4" t="n">
@@ -2737,7 +2737,7 @@
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>Week 4</t>
+          <t>Part 4</t>
         </is>
       </c>
       <c r="B70" s="4" t="n">
@@ -2770,7 +2770,7 @@
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>Week 4</t>
+          <t>Part 4</t>
         </is>
       </c>
       <c r="B71" s="4" t="n">
@@ -2803,7 +2803,7 @@
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>Week 4</t>
+          <t>Part 4</t>
         </is>
       </c>
       <c r="B72" s="4" t="n">
@@ -2836,7 +2836,7 @@
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>Week 4</t>
+          <t>Part 4</t>
         </is>
       </c>
       <c r="B73" s="4" t="n">
@@ -2869,7 +2869,7 @@
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>Week 4</t>
+          <t>Part 4</t>
         </is>
       </c>
       <c r="B74" s="4" t="n">
@@ -2902,7 +2902,7 @@
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>Week 4</t>
+          <t>Part 4</t>
         </is>
       </c>
       <c r="B75" s="4" t="n">
@@ -2935,7 +2935,7 @@
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>Week 4</t>
+          <t>Part 4</t>
         </is>
       </c>
       <c r="B76" s="4" t="n">
@@ -2968,7 +2968,7 @@
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>Week 4</t>
+          <t>Part 4</t>
         </is>
       </c>
       <c r="B77" s="4" t="n">
@@ -3001,7 +3001,7 @@
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>Week 4</t>
+          <t>Part 4</t>
         </is>
       </c>
       <c r="B78" s="4" t="n">
@@ -3034,7 +3034,7 @@
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>Week 4</t>
+          <t>Part 4</t>
         </is>
       </c>
       <c r="B79" s="4" t="n">
@@ -3067,7 +3067,7 @@
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>Week 4</t>
+          <t>Part 4</t>
         </is>
       </c>
       <c r="B80" s="4" t="n">
@@ -3100,14 +3100,14 @@
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
         <is>
-          <t>Week 5: Tone, Connotation &amp; Structure</t>
+          <t>Part 5: Tone, Connotation &amp; Structure</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>Week 5</t>
+          <t>Part 5</t>
         </is>
       </c>
       <c r="B82" s="4" t="n">
@@ -3140,7 +3140,7 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>Week 5</t>
+          <t>Part 5</t>
         </is>
       </c>
       <c r="B83" s="4" t="n">
@@ -3173,7 +3173,7 @@
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>Week 5</t>
+          <t>Part 5</t>
         </is>
       </c>
       <c r="B84" s="4" t="n">
@@ -3206,7 +3206,7 @@
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>Week 5</t>
+          <t>Part 5</t>
         </is>
       </c>
       <c r="B85" s="4" t="n">
@@ -3239,7 +3239,7 @@
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>Week 5</t>
+          <t>Part 5</t>
         </is>
       </c>
       <c r="B86" s="4" t="n">
@@ -3272,7 +3272,7 @@
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>Week 5</t>
+          <t>Part 5</t>
         </is>
       </c>
       <c r="B87" s="4" t="n">
@@ -3305,7 +3305,7 @@
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>Week 5</t>
+          <t>Part 5</t>
         </is>
       </c>
       <c r="B88" s="4" t="n">
@@ -3338,7 +3338,7 @@
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>Week 5</t>
+          <t>Part 5</t>
         </is>
       </c>
       <c r="B89" s="4" t="n">
@@ -3371,7 +3371,7 @@
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>Week 5</t>
+          <t>Part 5</t>
         </is>
       </c>
       <c r="B90" s="4" t="n">
@@ -3404,7 +3404,7 @@
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>Week 5</t>
+          <t>Part 5</t>
         </is>
       </c>
       <c r="B91" s="4" t="n">
@@ -3437,7 +3437,7 @@
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>Week 5</t>
+          <t>Part 5</t>
         </is>
       </c>
       <c r="B92" s="4" t="n">
@@ -3470,7 +3470,7 @@
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>Week 5</t>
+          <t>Part 5</t>
         </is>
       </c>
       <c r="B93" s="4" t="n">
@@ -3503,7 +3503,7 @@
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>Week 5</t>
+          <t>Part 5</t>
         </is>
       </c>
       <c r="B94" s="4" t="n">
@@ -3536,7 +3536,7 @@
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>Week 5</t>
+          <t>Part 5</t>
         </is>
       </c>
       <c r="B95" s="4" t="n">
@@ -3569,7 +3569,7 @@
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>Week 5</t>
+          <t>Part 5</t>
         </is>
       </c>
       <c r="B96" s="4" t="n">
@@ -3602,7 +3602,7 @@
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>Week 5</t>
+          <t>Part 5</t>
         </is>
       </c>
       <c r="B97" s="4" t="n">
@@ -3635,7 +3635,7 @@
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>Week 5</t>
+          <t>Part 5</t>
         </is>
       </c>
       <c r="B98" s="4" t="n">
@@ -3668,7 +3668,7 @@
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>Week 5</t>
+          <t>Part 5</t>
         </is>
       </c>
       <c r="B99" s="4" t="n">
@@ -3701,7 +3701,7 @@
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
         <is>
-          <t>Week 5</t>
+          <t>Part 5</t>
         </is>
       </c>
       <c r="B100" s="4" t="n">
@@ -3734,7 +3734,7 @@
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>Week 5</t>
+          <t>Part 5</t>
         </is>
       </c>
       <c r="B101" s="4" t="n">
@@ -3767,14 +3767,14 @@
     <row r="102">
       <c r="A102" s="9" t="inlineStr">
         <is>
-          <t>Week 6: Cross-Text Comparison &amp; Synthesis</t>
+          <t>Part 6: Cross-Text Comparison &amp; Synthesis</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>Week 6</t>
+          <t>Part 6</t>
         </is>
       </c>
       <c r="B103" s="4" t="n">
@@ -3807,7 +3807,7 @@
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
         <is>
-          <t>Week 6</t>
+          <t>Part 6</t>
         </is>
       </c>
       <c r="B104" s="4" t="n">
@@ -3840,7 +3840,7 @@
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t>Week 6</t>
+          <t>Part 6</t>
         </is>
       </c>
       <c r="B105" s="4" t="n">
@@ -3873,7 +3873,7 @@
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t>Week 6</t>
+          <t>Part 6</t>
         </is>
       </c>
       <c r="B106" s="4" t="n">
@@ -3906,7 +3906,7 @@
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>Week 6</t>
+          <t>Part 6</t>
         </is>
       </c>
       <c r="B107" s="4" t="n">
@@ -3939,7 +3939,7 @@
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>Week 6</t>
+          <t>Part 6</t>
         </is>
       </c>
       <c r="B108" s="4" t="n">
@@ -3972,7 +3972,7 @@
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>Week 6</t>
+          <t>Part 6</t>
         </is>
       </c>
       <c r="B109" s="4" t="n">
@@ -4005,7 +4005,7 @@
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>Week 6</t>
+          <t>Part 6</t>
         </is>
       </c>
       <c r="B110" s="4" t="n">
@@ -4038,7 +4038,7 @@
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>Week 6</t>
+          <t>Part 6</t>
         </is>
       </c>
       <c r="B111" s="4" t="n">
@@ -4071,7 +4071,7 @@
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>Week 6</t>
+          <t>Part 6</t>
         </is>
       </c>
       <c r="B112" s="4" t="n">
@@ -4104,7 +4104,7 @@
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>Week 6</t>
+          <t>Part 6</t>
         </is>
       </c>
       <c r="B113" s="4" t="n">
@@ -4137,7 +4137,7 @@
     <row r="114">
       <c r="A114" s="3" t="inlineStr">
         <is>
-          <t>Week 6</t>
+          <t>Part 6</t>
         </is>
       </c>
       <c r="B114" s="4" t="n">
@@ -4170,7 +4170,7 @@
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>Week 6</t>
+          <t>Part 6</t>
         </is>
       </c>
       <c r="B115" s="4" t="n">
@@ -4203,7 +4203,7 @@
     <row r="116">
       <c r="A116" s="3" t="inlineStr">
         <is>
-          <t>Week 6</t>
+          <t>Part 6</t>
         </is>
       </c>
       <c r="B116" s="4" t="n">
@@ -4236,7 +4236,7 @@
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
         <is>
-          <t>Week 6</t>
+          <t>Part 6</t>
         </is>
       </c>
       <c r="B117" s="4" t="n">
@@ -4266,6 +4266,7 @@
         </is>
       </c>
     </row>
+    <row r="118"/>
     <row r="119">
       <c r="A119" s="10" t="inlineStr">
         <is>
@@ -4317,6 +4318,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
@@ -4361,7 +4363,7 @@
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>6 weeks</t>
+          <t>6 parts</t>
         </is>
       </c>
     </row>
@@ -4377,10 +4379,11 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>Week</t>
+          <t>Part</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -4402,7 +4405,7 @@
     <row r="10">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t>Week 1</t>
+          <t>Part 1</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
@@ -4420,7 +4423,7 @@
     <row r="11">
       <c r="A11" s="17" t="inlineStr">
         <is>
-          <t>Week 2</t>
+          <t>Part 2</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
@@ -4438,7 +4441,7 @@
     <row r="12">
       <c r="A12" s="18" t="inlineStr">
         <is>
-          <t>Week 3</t>
+          <t>Part 3</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -4456,7 +4459,7 @@
     <row r="13">
       <c r="A13" s="19" t="inlineStr">
         <is>
-          <t>Week 4</t>
+          <t>Part 4</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
@@ -4474,7 +4477,7 @@
     <row r="14">
       <c r="A14" s="20" t="inlineStr">
         <is>
-          <t>Week 5</t>
+          <t>Part 5</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
@@ -4492,7 +4495,7 @@
     <row r="15">
       <c r="A15" s="21" t="inlineStr">
         <is>
-          <t>Week 6</t>
+          <t>Part 6</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">

</xml_diff>